<commit_message>
v0.3.5 - Fix: GEO_BLOCKED erweitert + Südbaden-Bug + functions.schema aktualisiert
</commit_message>
<xml_diff>
--- a/Liga-Zuordnungen.xlsx
+++ b/Liga-Zuordnungen.xlsx
@@ -699,126 +699,126 @@
       <c r="I5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>einzeln</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>geo_gesperrt</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>6-14</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Landesliga Weser-Ems</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" s="5" t="n">
+      <c r="E6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>fix gesperrt (kein SIBLING_GROUPS-Eintrag)</t>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Keyword: Weser-Ems</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>einzeln</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>geo_gesperrt</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>6-15</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Landesliga Lüneburg</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="5" t="n">
+      <c r="E7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>fix gesperrt (kein SIBLING_GROUPS-Eintrag)</t>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Keyword: Lüneburg</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>einzeln</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>geo_gesperrt</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>6-16</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Landesliga Hannover</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="5" t="n">
+      <c r="E8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>fix gesperrt (kein SIBLING_GROUPS-Eintrag)</t>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Keyword: Hannover</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>einzeln</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>geo_gesperrt</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>6-17</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Landesliga Braunschweig</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="5" t="n">
+      <c r="E9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>fix gesperrt (kein SIBLING_GROUPS-Eintrag)</t>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Keyword: Braunschweig</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2022,7 @@
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Keyword: Baden</t>
+          <t>Keyword: Südbaden (Fix: war Baden, false-negative)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.3.9 - Fix: Routing-Korrekturen Südwest + Hessen
</commit_message>
<xml_diff>
--- a/Liga-Zuordnungen.xlsx
+++ b/Liga-Zuordnungen.xlsx
@@ -2078,7 +2078,7 @@
         <v>6</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
       <c r="H47" s="4" t="inlineStr"/>
@@ -2109,7 +2109,7 @@
         <v>6</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
       <c r="H48" s="4" t="inlineStr"/>
@@ -2140,7 +2140,7 @@
         <v>6</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr"/>

</xml_diff>